<commit_message>
Aggiornamento storico e simulazione (Fase Post-Match)
</commit_message>
<xml_diff>
--- a/Storico_Validato_Betting.xlsx
+++ b/Storico_Validato_Betting.xlsx
@@ -14,7 +14,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="327" uniqueCount="77">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="344" uniqueCount="74">
   <si>
     <t>Campionato</t>
   </si>
@@ -73,13 +73,16 @@
     <t>U/O 2.5</t>
   </si>
   <si>
-    <t>Risultato Reale</t>
-  </si>
-  <si>
-    <t>Esito 1X2</t>
-  </si>
-  <si>
-    <t>Esito U/O 2.5</t>
+    <t>Risultato_Reale</t>
+  </si>
+  <si>
+    <t>Esito_1X2</t>
+  </si>
+  <si>
+    <t>Esito_Risultato_Esatto</t>
+  </si>
+  <si>
+    <t>Esito_U/O_2.5</t>
   </si>
   <si>
     <t>Esito DC+U/O2.5</t>
@@ -223,19 +226,7 @@
     <t>3-1</t>
   </si>
   <si>
-    <t>In Attesa</t>
-  </si>
-  <si>
-    <t>2-0</t>
-  </si>
-  <si>
-    <t>4-1</t>
-  </si>
-  <si>
-    <t>2-2</t>
-  </si>
-  <si>
-    <t>7-1</t>
+    <t>NON ANCORA REALE/DA VALIDARE</t>
   </si>
   <si>
     <t>VINCENTE</t>
@@ -602,10 +593,10 @@
 
 <file path=xl/worksheets/sheet1.xml><?xml version="1.0" encoding="utf-8"?>
 <worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships">
-  <dimension ref="A1:W17"/>
+  <dimension ref="A1:X17"/>
   <sheetFormatPr defaultRowHeight="15"/>
   <sheetData>
-    <row r="1" spans="1:23">
+    <row r="1" spans="1:24">
       <c r="A1" s="1" t="s">
         <v>0</v>
       </c>
@@ -675,16 +666,19 @@
       <c r="W1" s="1" t="s">
         <v>22</v>
       </c>
+      <c r="X1" s="1" t="s">
+        <v>23</v>
+      </c>
     </row>
-    <row r="2" spans="1:23">
+    <row r="2" spans="1:24">
       <c r="A2" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B2" t="s">
-        <v>24</v>
+        <v>25</v>
       </c>
       <c r="C2" t="s">
-        <v>40</v>
+        <v>41</v>
       </c>
       <c r="D2">
         <v>0</v>
@@ -693,69 +687,72 @@
         <v>0</v>
       </c>
       <c r="F2" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G2" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H2">
         <v>1</v>
       </c>
       <c r="I2" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J2" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K2" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M2" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N2" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O2" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P2" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q2" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R2">
         <v>1</v>
       </c>
       <c r="S2" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T2" t="s">
-        <v>67</v>
+        <v>68</v>
       </c>
       <c r="U2" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="V2" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="W2" t="s">
-        <v>76</v>
+        <v>73</v>
+      </c>
+      <c r="X2" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="3" spans="1:23">
+    <row r="3" spans="1:24">
       <c r="A3" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B3" t="s">
-        <v>25</v>
+        <v>26</v>
       </c>
       <c r="C3" t="s">
-        <v>41</v>
+        <v>42</v>
       </c>
       <c r="D3">
         <v>0</v>
@@ -764,69 +761,72 @@
         <v>0</v>
       </c>
       <c r="F3" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G3" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H3">
         <v>1</v>
       </c>
       <c r="I3" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J3" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K3" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M3" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N3" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O3" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P3" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q3" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R3">
         <v>1</v>
       </c>
       <c r="S3" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T3" t="s">
-        <v>68</v>
+        <v>69</v>
       </c>
       <c r="U3" t="s">
-        <v>74</v>
+        <v>71</v>
       </c>
       <c r="V3" t="s">
-        <v>76</v>
+        <v>73</v>
       </c>
       <c r="W3" t="s">
-        <v>76</v>
+        <v>73</v>
+      </c>
+      <c r="X3" t="s">
+        <v>73</v>
       </c>
     </row>
-    <row r="4" spans="1:23">
+    <row r="4" spans="1:24">
       <c r="A4" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B4" t="s">
-        <v>26</v>
+        <v>27</v>
       </c>
       <c r="C4" t="s">
-        <v>42</v>
+        <v>43</v>
       </c>
       <c r="D4">
         <v>0</v>
@@ -835,69 +835,72 @@
         <v>0</v>
       </c>
       <c r="F4" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G4" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H4">
         <v>1</v>
       </c>
       <c r="I4" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J4" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K4" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M4" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N4" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O4" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P4" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q4" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R4">
         <v>1</v>
       </c>
       <c r="S4" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T4" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V4" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W4" t="s">
-        <v>75</v>
+        <v>72</v>
+      </c>
+      <c r="X4" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="5" spans="1:23">
+    <row r="5" spans="1:24">
       <c r="A5" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B5" t="s">
-        <v>27</v>
+        <v>28</v>
       </c>
       <c r="C5" t="s">
-        <v>43</v>
+        <v>44</v>
       </c>
       <c r="D5">
         <v>0</v>
@@ -906,69 +909,72 @@
         <v>0</v>
       </c>
       <c r="F5" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G5" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H5">
         <v>1</v>
       </c>
       <c r="I5" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J5" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K5" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M5" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N5" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O5" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P5" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q5" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R5">
         <v>1</v>
       </c>
       <c r="S5" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T5" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V5" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W5" t="s">
-        <v>75</v>
+        <v>72</v>
+      </c>
+      <c r="X5" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="6" spans="1:23">
+    <row r="6" spans="1:24">
       <c r="A6" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B6" t="s">
-        <v>28</v>
+        <v>29</v>
       </c>
       <c r="C6" t="s">
-        <v>44</v>
+        <v>45</v>
       </c>
       <c r="D6">
         <v>0</v>
@@ -977,69 +983,72 @@
         <v>0</v>
       </c>
       <c r="F6" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G6" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H6">
         <v>1</v>
       </c>
       <c r="I6" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J6" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K6" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M6" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N6" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O6" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P6" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q6" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R6">
         <v>1</v>
       </c>
       <c r="S6" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T6" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V6" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W6" t="s">
-        <v>75</v>
+        <v>72</v>
+      </c>
+      <c r="X6" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="7" spans="1:23">
+    <row r="7" spans="1:24">
       <c r="A7" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B7" t="s">
-        <v>29</v>
+        <v>30</v>
       </c>
       <c r="C7" t="s">
-        <v>45</v>
+        <v>46</v>
       </c>
       <c r="D7">
         <v>0</v>
@@ -1048,69 +1057,72 @@
         <v>0</v>
       </c>
       <c r="F7" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G7" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H7">
         <v>1</v>
       </c>
       <c r="I7" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J7" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K7" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M7" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N7" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O7" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P7" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q7" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R7">
         <v>1</v>
       </c>
       <c r="S7" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T7" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V7" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W7" t="s">
-        <v>75</v>
+        <v>72</v>
+      </c>
+      <c r="X7" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="8" spans="1:23">
+    <row r="8" spans="1:24">
       <c r="A8" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B8" t="s">
-        <v>30</v>
+        <v>31</v>
       </c>
       <c r="C8" t="s">
-        <v>46</v>
+        <v>47</v>
       </c>
       <c r="D8">
         <v>0</v>
@@ -1119,211 +1131,220 @@
         <v>0</v>
       </c>
       <c r="F8" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G8" t="s">
+        <v>58</v>
+      </c>
+      <c r="H8">
+        <v>1</v>
+      </c>
+      <c r="I8" t="s">
+        <v>59</v>
+      </c>
+      <c r="J8" t="s">
+        <v>60</v>
+      </c>
+      <c r="K8" t="s">
+        <v>61</v>
+      </c>
+      <c r="L8" t="s">
+        <v>62</v>
+      </c>
+      <c r="M8" t="s">
+        <v>63</v>
+      </c>
+      <c r="N8" t="s">
+        <v>64</v>
+      </c>
+      <c r="O8" t="s">
+        <v>65</v>
+      </c>
+      <c r="P8" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q8" t="s">
+        <v>67</v>
+      </c>
+      <c r="R8">
+        <v>1</v>
+      </c>
+      <c r="S8" t="s">
+        <v>62</v>
+      </c>
+      <c r="T8" t="s">
+        <v>70</v>
+      </c>
+      <c r="U8" t="s">
+        <v>72</v>
+      </c>
+      <c r="V8" t="s">
+        <v>72</v>
+      </c>
+      <c r="W8" t="s">
+        <v>72</v>
+      </c>
+      <c r="X8" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="9" spans="1:24">
+      <c r="A9" t="s">
+        <v>24</v>
+      </c>
+      <c r="B9" t="s">
+        <v>32</v>
+      </c>
+      <c r="C9" t="s">
+        <v>48</v>
+      </c>
+      <c r="D9">
+        <v>1</v>
+      </c>
+      <c r="E9">
+        <v>1</v>
+      </c>
+      <c r="F9" t="s">
         <v>57</v>
       </c>
-      <c r="H8">
-        <v>1</v>
-      </c>
-      <c r="I8" t="s">
+      <c r="G9" t="s">
         <v>58</v>
       </c>
-      <c r="J8" t="s">
+      <c r="H9">
+        <v>1</v>
+      </c>
+      <c r="I9" t="s">
         <v>59</v>
       </c>
-      <c r="K8" t="s">
+      <c r="J9" t="s">
         <v>60</v>
       </c>
-      <c r="L8" t="s">
+      <c r="K9" t="s">
         <v>61</v>
       </c>
-      <c r="M8" t="s">
-        <v>62</v>
-      </c>
-      <c r="N8" t="s">
+      <c r="L9" t="s">
+        <v>62</v>
+      </c>
+      <c r="M9" t="s">
         <v>63</v>
       </c>
-      <c r="O8" t="s">
+      <c r="N9" t="s">
         <v>64</v>
       </c>
-      <c r="P8" t="s">
+      <c r="O9" t="s">
         <v>65</v>
       </c>
-      <c r="Q8" t="s">
+      <c r="P9" t="s">
         <v>66</v>
       </c>
-      <c r="R8">
-        <v>1</v>
-      </c>
-      <c r="S8" t="s">
+      <c r="Q9" t="s">
+        <v>67</v>
+      </c>
+      <c r="R9">
+        <v>1</v>
+      </c>
+      <c r="S9" t="s">
+        <v>62</v>
+      </c>
+      <c r="T9" t="s">
+        <v>70</v>
+      </c>
+      <c r="U9" t="s">
+        <v>72</v>
+      </c>
+      <c r="V9" t="s">
+        <v>72</v>
+      </c>
+      <c r="W9" t="s">
+        <v>72</v>
+      </c>
+      <c r="X9" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="10" spans="1:24">
+      <c r="A10" t="s">
+        <v>24</v>
+      </c>
+      <c r="B10" t="s">
+        <v>33</v>
+      </c>
+      <c r="C10" t="s">
+        <v>49</v>
+      </c>
+      <c r="D10">
+        <v>1</v>
+      </c>
+      <c r="E10">
+        <v>1</v>
+      </c>
+      <c r="F10" t="s">
+        <v>57</v>
+      </c>
+      <c r="G10" t="s">
+        <v>58</v>
+      </c>
+      <c r="H10">
+        <v>1</v>
+      </c>
+      <c r="I10" t="s">
+        <v>59</v>
+      </c>
+      <c r="J10" t="s">
+        <v>60</v>
+      </c>
+      <c r="K10" t="s">
         <v>61</v>
       </c>
-      <c r="T8" t="s">
-        <v>69</v>
-      </c>
-      <c r="U8" t="s">
-        <v>75</v>
-      </c>
-      <c r="V8" t="s">
-        <v>75</v>
-      </c>
-      <c r="W8" t="s">
-        <v>75</v>
+      <c r="L10" t="s">
+        <v>62</v>
+      </c>
+      <c r="M10" t="s">
+        <v>63</v>
+      </c>
+      <c r="N10" t="s">
+        <v>64</v>
+      </c>
+      <c r="O10" t="s">
+        <v>65</v>
+      </c>
+      <c r="P10" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q10" t="s">
+        <v>67</v>
+      </c>
+      <c r="R10">
+        <v>1</v>
+      </c>
+      <c r="S10" t="s">
+        <v>62</v>
+      </c>
+      <c r="T10" t="s">
+        <v>70</v>
+      </c>
+      <c r="U10" t="s">
+        <v>72</v>
+      </c>
+      <c r="V10" t="s">
+        <v>72</v>
+      </c>
+      <c r="W10" t="s">
+        <v>72</v>
+      </c>
+      <c r="X10" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="9" spans="1:23">
-      <c r="A9" t="s">
-        <v>23</v>
-      </c>
-      <c r="B9" t="s">
-        <v>31</v>
-      </c>
-      <c r="C9" t="s">
-        <v>47</v>
-      </c>
-      <c r="D9">
-        <v>1</v>
-      </c>
-      <c r="E9">
-        <v>1</v>
-      </c>
-      <c r="F9" t="s">
-        <v>56</v>
-      </c>
-      <c r="G9" t="s">
-        <v>57</v>
-      </c>
-      <c r="H9">
-        <v>1</v>
-      </c>
-      <c r="I9" t="s">
-        <v>58</v>
-      </c>
-      <c r="J9" t="s">
-        <v>59</v>
-      </c>
-      <c r="K9" t="s">
-        <v>60</v>
-      </c>
-      <c r="L9" t="s">
-        <v>61</v>
-      </c>
-      <c r="M9" t="s">
-        <v>62</v>
-      </c>
-      <c r="N9" t="s">
-        <v>63</v>
-      </c>
-      <c r="O9" t="s">
-        <v>64</v>
-      </c>
-      <c r="P9" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q9" t="s">
-        <v>66</v>
-      </c>
-      <c r="R9">
-        <v>1</v>
-      </c>
-      <c r="S9" t="s">
-        <v>61</v>
-      </c>
-      <c r="T9" t="s">
-        <v>69</v>
-      </c>
-      <c r="U9" t="s">
-        <v>75</v>
-      </c>
-      <c r="V9" t="s">
-        <v>75</v>
-      </c>
-      <c r="W9" t="s">
-        <v>75</v>
-      </c>
-    </row>
-    <row r="10" spans="1:23">
-      <c r="A10" t="s">
-        <v>23</v>
-      </c>
-      <c r="B10" t="s">
-        <v>32</v>
-      </c>
-      <c r="C10" t="s">
-        <v>48</v>
-      </c>
-      <c r="D10">
-        <v>1</v>
-      </c>
-      <c r="E10">
-        <v>1</v>
-      </c>
-      <c r="F10" t="s">
-        <v>56</v>
-      </c>
-      <c r="G10" t="s">
-        <v>57</v>
-      </c>
-      <c r="H10">
-        <v>1</v>
-      </c>
-      <c r="I10" t="s">
-        <v>58</v>
-      </c>
-      <c r="J10" t="s">
-        <v>59</v>
-      </c>
-      <c r="K10" t="s">
-        <v>60</v>
-      </c>
-      <c r="L10" t="s">
-        <v>61</v>
-      </c>
-      <c r="M10" t="s">
-        <v>62</v>
-      </c>
-      <c r="N10" t="s">
-        <v>63</v>
-      </c>
-      <c r="O10" t="s">
-        <v>64</v>
-      </c>
-      <c r="P10" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q10" t="s">
-        <v>66</v>
-      </c>
-      <c r="R10">
-        <v>1</v>
-      </c>
-      <c r="S10" t="s">
-        <v>61</v>
-      </c>
-      <c r="T10" t="s">
-        <v>58</v>
-      </c>
-      <c r="U10" t="s">
-        <v>76</v>
-      </c>
-      <c r="V10" t="s">
-        <v>74</v>
-      </c>
-      <c r="W10" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="11" spans="1:23">
+    <row r="11" spans="1:24">
       <c r="A11" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B11" t="s">
-        <v>33</v>
+        <v>34</v>
       </c>
       <c r="C11" t="s">
-        <v>49</v>
+        <v>50</v>
       </c>
       <c r="D11">
         <v>3</v>
@@ -1332,69 +1353,72 @@
         <v>3</v>
       </c>
       <c r="F11" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G11" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H11">
         <v>1</v>
       </c>
       <c r="I11" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J11" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K11" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M11" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N11" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O11" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P11" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q11" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R11">
         <v>1</v>
       </c>
       <c r="S11" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T11" t="s">
         <v>70</v>
       </c>
       <c r="U11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="V11" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="W11" t="s">
-        <v>76</v>
+        <v>72</v>
+      </c>
+      <c r="X11" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="12" spans="1:23">
+    <row r="12" spans="1:24">
       <c r="A12" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B12" t="s">
-        <v>34</v>
+        <v>35</v>
       </c>
       <c r="C12" t="s">
-        <v>50</v>
+        <v>51</v>
       </c>
       <c r="D12">
         <v>3</v>
@@ -1403,69 +1427,72 @@
         <v>3</v>
       </c>
       <c r="F12" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G12" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H12">
         <v>1</v>
       </c>
       <c r="I12" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J12" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K12" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M12" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N12" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O12" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P12" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q12" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R12">
         <v>1</v>
       </c>
       <c r="S12" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T12" t="s">
-        <v>71</v>
+        <v>70</v>
       </c>
       <c r="U12" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="V12" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="W12" t="s">
-        <v>76</v>
+        <v>72</v>
+      </c>
+      <c r="X12" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="13" spans="1:23">
+    <row r="13" spans="1:24">
       <c r="A13" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B13" t="s">
-        <v>35</v>
+        <v>36</v>
       </c>
       <c r="C13" t="s">
-        <v>51</v>
+        <v>52</v>
       </c>
       <c r="D13">
         <v>3</v>
@@ -1474,69 +1501,72 @@
         <v>1</v>
       </c>
       <c r="F13" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G13" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H13">
         <v>1</v>
       </c>
       <c r="I13" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J13" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K13" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M13" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N13" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O13" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P13" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q13" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R13">
         <v>1</v>
       </c>
       <c r="S13" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T13" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V13" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W13" t="s">
-        <v>75</v>
+        <v>72</v>
+      </c>
+      <c r="X13" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="14" spans="1:23">
+    <row r="14" spans="1:24">
       <c r="A14" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B14" t="s">
-        <v>36</v>
+        <v>37</v>
       </c>
       <c r="C14" t="s">
-        <v>52</v>
+        <v>53</v>
       </c>
       <c r="D14">
         <v>1</v>
@@ -1545,69 +1575,72 @@
         <v>0</v>
       </c>
       <c r="F14" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G14" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H14">
         <v>1</v>
       </c>
       <c r="I14" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J14" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K14" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M14" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N14" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O14" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P14" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q14" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R14">
         <v>1</v>
       </c>
       <c r="S14" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T14" t="s">
-        <v>58</v>
+        <v>70</v>
       </c>
       <c r="U14" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="V14" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="W14" t="s">
-        <v>76</v>
+        <v>72</v>
+      </c>
+      <c r="X14" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="15" spans="1:23">
+    <row r="15" spans="1:24">
       <c r="A15" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B15" t="s">
-        <v>37</v>
+        <v>38</v>
       </c>
       <c r="C15" t="s">
-        <v>53</v>
+        <v>54</v>
       </c>
       <c r="D15">
         <v>0</v>
@@ -1616,69 +1649,72 @@
         <v>0</v>
       </c>
       <c r="F15" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G15" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H15">
         <v>1</v>
       </c>
       <c r="I15" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J15" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K15" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M15" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N15" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O15" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P15" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q15" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R15">
         <v>1</v>
       </c>
       <c r="S15" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T15" t="s">
-        <v>69</v>
+        <v>70</v>
       </c>
       <c r="U15" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="V15" t="s">
-        <v>75</v>
+        <v>72</v>
       </c>
       <c r="W15" t="s">
-        <v>75</v>
+        <v>72</v>
+      </c>
+      <c r="X15" t="s">
+        <v>72</v>
       </c>
     </row>
-    <row r="16" spans="1:23">
+    <row r="16" spans="1:24">
       <c r="A16" t="s">
-        <v>23</v>
+        <v>24</v>
       </c>
       <c r="B16" t="s">
-        <v>38</v>
+        <v>39</v>
       </c>
       <c r="C16" t="s">
-        <v>54</v>
+        <v>55</v>
       </c>
       <c r="D16">
         <v>1</v>
@@ -1687,69 +1723,72 @@
         <v>3</v>
       </c>
       <c r="F16" t="s">
+        <v>57</v>
+      </c>
+      <c r="G16" t="s">
+        <v>58</v>
+      </c>
+      <c r="H16">
+        <v>1</v>
+      </c>
+      <c r="I16" t="s">
+        <v>59</v>
+      </c>
+      <c r="J16" t="s">
+        <v>60</v>
+      </c>
+      <c r="K16" t="s">
+        <v>61</v>
+      </c>
+      <c r="L16" t="s">
+        <v>62</v>
+      </c>
+      <c r="M16" t="s">
+        <v>63</v>
+      </c>
+      <c r="N16" t="s">
+        <v>64</v>
+      </c>
+      <c r="O16" t="s">
+        <v>65</v>
+      </c>
+      <c r="P16" t="s">
+        <v>66</v>
+      </c>
+      <c r="Q16" t="s">
+        <v>67</v>
+      </c>
+      <c r="R16">
+        <v>1</v>
+      </c>
+      <c r="S16" t="s">
+        <v>62</v>
+      </c>
+      <c r="T16" t="s">
+        <v>70</v>
+      </c>
+      <c r="U16" t="s">
+        <v>72</v>
+      </c>
+      <c r="V16" t="s">
+        <v>72</v>
+      </c>
+      <c r="W16" t="s">
+        <v>72</v>
+      </c>
+      <c r="X16" t="s">
+        <v>72</v>
+      </c>
+    </row>
+    <row r="17" spans="1:24">
+      <c r="A17" t="s">
+        <v>24</v>
+      </c>
+      <c r="B17" t="s">
+        <v>40</v>
+      </c>
+      <c r="C17" t="s">
         <v>56</v>
-      </c>
-      <c r="G16" t="s">
-        <v>57</v>
-      </c>
-      <c r="H16">
-        <v>1</v>
-      </c>
-      <c r="I16" t="s">
-        <v>58</v>
-      </c>
-      <c r="J16" t="s">
-        <v>59</v>
-      </c>
-      <c r="K16" t="s">
-        <v>60</v>
-      </c>
-      <c r="L16" t="s">
-        <v>61</v>
-      </c>
-      <c r="M16" t="s">
-        <v>62</v>
-      </c>
-      <c r="N16" t="s">
-        <v>63</v>
-      </c>
-      <c r="O16" t="s">
-        <v>64</v>
-      </c>
-      <c r="P16" t="s">
-        <v>65</v>
-      </c>
-      <c r="Q16" t="s">
-        <v>66</v>
-      </c>
-      <c r="R16">
-        <v>1</v>
-      </c>
-      <c r="S16" t="s">
-        <v>61</v>
-      </c>
-      <c r="T16" t="s">
-        <v>72</v>
-      </c>
-      <c r="U16" t="s">
-        <v>76</v>
-      </c>
-      <c r="V16" t="s">
-        <v>76</v>
-      </c>
-      <c r="W16" t="s">
-        <v>76</v>
-      </c>
-    </row>
-    <row r="17" spans="1:23">
-      <c r="A17" t="s">
-        <v>23</v>
-      </c>
-      <c r="B17" t="s">
-        <v>39</v>
-      </c>
-      <c r="C17" t="s">
-        <v>55</v>
       </c>
       <c r="D17">
         <v>3</v>
@@ -1758,58 +1797,61 @@
         <v>3</v>
       </c>
       <c r="F17" t="s">
-        <v>56</v>
+        <v>57</v>
       </c>
       <c r="G17" t="s">
-        <v>57</v>
+        <v>58</v>
       </c>
       <c r="H17">
         <v>1</v>
       </c>
       <c r="I17" t="s">
-        <v>58</v>
+        <v>59</v>
       </c>
       <c r="J17" t="s">
-        <v>59</v>
+        <v>60</v>
       </c>
       <c r="K17" t="s">
-        <v>60</v>
+        <v>61</v>
       </c>
       <c r="L17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="M17" t="s">
-        <v>62</v>
+        <v>63</v>
       </c>
       <c r="N17" t="s">
-        <v>63</v>
+        <v>64</v>
       </c>
       <c r="O17" t="s">
-        <v>64</v>
+        <v>65</v>
       </c>
       <c r="P17" t="s">
-        <v>65</v>
+        <v>66</v>
       </c>
       <c r="Q17" t="s">
-        <v>66</v>
+        <v>67</v>
       </c>
       <c r="R17">
         <v>1</v>
       </c>
       <c r="S17" t="s">
-        <v>61</v>
+        <v>62</v>
       </c>
       <c r="T17" t="s">
-        <v>73</v>
+        <v>70</v>
       </c>
       <c r="U17" t="s">
-        <v>74</v>
+        <v>72</v>
       </c>
       <c r="V17" t="s">
-        <v>76</v>
+        <v>72</v>
       </c>
       <c r="W17" t="s">
-        <v>76</v>
+        <v>72</v>
+      </c>
+      <c r="X17" t="s">
+        <v>72</v>
       </c>
     </row>
   </sheetData>

</xml_diff>